<commit_message>
Add user auth, OTP forgot password, email service, and pytest test suite
</commit_message>
<xml_diff>
--- a/financial_report.xlsx
+++ b/financial_report.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Budget" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Expenses" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,6 +495,31 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>aug</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sep salary</t>
         </is>
       </c>
     </row>
@@ -507,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,6 +586,31 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>enjoyed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>movies</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>upi</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sep</t>
         </is>
       </c>
     </row>
@@ -573,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,6 +648,16 @@
       </c>
       <c r="B2" t="n">
         <v>3000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
@@ -609,6 +671,248 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>sep salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>900</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>movies</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>upi</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>aug</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>upi</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>enjoyed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>job</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>aug salary</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>movies</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>900</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -631,7 +935,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="3">
@@ -641,7 +945,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1200</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="4">
@@ -651,17 +955,17 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3800</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Current Budget</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>